<commit_message>
Dashboard: 2026-09-01 14:23 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/resumo_macro.xlsx
+++ b/greenlife_scraper/resumo_macro.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1006,6 +1006,24 @@
         <v>200</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n">
+        <v>249583</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1269</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>